<commit_message>
chore: remove unnecessary trailing spaces in endpoint file
(note: code has been updated to remove trailing spaces from fields in the dataframe when loaded, but the file itself has been updated as well)
</commit_message>
<xml_diff>
--- a/data/SuperEndpoint Mapping 2025NOV20.xlsx
+++ b/data/SuperEndpoint Mapping 2025NOV20.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pnnl-my.sharepoint.com/personal/christine_chang_pnnl_gov/Documents/Documents/Projects/superfund/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pnnl-my.sharepoint.com/personal/christine_chang_pnnl_gov/Documents/Documents/Projects/superfund/repos/srpAnalytics/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A73875D4-5097-FC4E-B3CC-5136622899C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="8_{A73875D4-5097-FC4E-B3CC-5136622899C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD9A4D8B-8D21-9A4D-A770-19701077373A}"/>
   <bookViews>
-    <workbookView xWindow="20080" yWindow="11720" windowWidth="23460" windowHeight="17060" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1420" yWindow="9120" windowWidth="37300" windowHeight="18620" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Original" sheetId="4" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="239">
   <si>
     <t>New Endpoints</t>
   </si>
@@ -202,36 +202,12 @@
     <t>ANY24</t>
   </si>
   <si>
-    <t>ANY120  </t>
-  </si>
-  <si>
     <t>TOT_MORT</t>
   </si>
   <si>
-    <t>BRN_    </t>
-  </si>
-  <si>
-    <t>CRAN    </t>
-  </si>
-  <si>
-    <t>EDEM    </t>
-  </si>
-  <si>
-    <t>MUSC    </t>
-  </si>
-  <si>
-    <t>SKIN    </t>
-  </si>
-  <si>
-    <t>TCHR   </t>
-  </si>
-  <si>
     <t>MOV1</t>
   </si>
   <si>
-    <t>AUC1 </t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -433,18 +409,12 @@
     <t>name</t>
   </si>
   <si>
-    <t>cardiovascular system</t>
-  </si>
-  <si>
     <t>ZFA:0000010</t>
   </si>
   <si>
     <t>ZFA:0000107</t>
   </si>
   <si>
-    <t>pericardial cavity</t>
-  </si>
-  <si>
     <t>ZFA:0005496</t>
   </si>
   <si>
@@ -661,12 +631,6 @@
     <t>http://purl.obolibrary.org/obo/ZP_0000100</t>
   </si>
   <si>
-    <t>otic vesicle morphology, abnormal</t>
-  </si>
-  <si>
-    <t>pectoral fin physical object quality, abnormal</t>
-  </si>
-  <si>
     <t>http://purl.obolibrary.org/obo/ZP_0000943</t>
   </si>
   <si>
@@ -718,10 +682,70 @@
     <t>ZFA:0000054</t>
   </si>
   <si>
-    <t>bent body axis</t>
-  </si>
-  <si>
     <t>ZFA:0001227</t>
+  </si>
+  <si>
+    <t>AUC</t>
+  </si>
+  <si>
+    <t>MOV</t>
+  </si>
+  <si>
+    <t>Pericardial cavity</t>
+  </si>
+  <si>
+    <t>Lower trunk</t>
+  </si>
+  <si>
+    <t>Caudal fin</t>
+  </si>
+  <si>
+    <t>Cardiovascular system</t>
+  </si>
+  <si>
+    <t>Bent body axis</t>
+  </si>
+  <si>
+    <t>Eye</t>
+  </si>
+  <si>
+    <t>Jaw</t>
+  </si>
+  <si>
+    <t>Yolk sac edema</t>
+  </si>
+  <si>
+    <t>Otic vesicle morphology, abnormal</t>
+  </si>
+  <si>
+    <t>Pectoral fin physical object quality, abnormal</t>
+  </si>
+  <si>
+    <t>Snout</t>
+  </si>
+  <si>
+    <t>Pigmentation</t>
+  </si>
+  <si>
+    <t>Somite</t>
+  </si>
+  <si>
+    <t>Swim bladder inflation</t>
+  </si>
+  <si>
+    <t>Touch response</t>
+  </si>
+  <si>
+    <t>Trunk</t>
+  </si>
+  <si>
+    <t>ANY120</t>
+  </si>
+  <si>
+    <t>AUC1</t>
+  </si>
+  <si>
+    <t>BRN_</t>
   </si>
 </sst>
 </file>
@@ -1211,13 +1235,13 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -1225,10 +1249,10 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1236,10 +1260,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1247,10 +1271,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -1258,21 +1282,21 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1280,21 +1304,21 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1302,10 +1326,10 @@
         <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -1313,43 +1337,43 @@
         <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C12" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B13" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1357,10 +1381,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -1368,43 +1392,43 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C15" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B17" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B18" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -1412,43 +1436,43 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C19" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C20" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B21" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C21" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B22" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1756,7 +1780,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0498EF9C-E9A3-468C-A290-DEE17D385575}">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
@@ -1766,568 +1790,613 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D1" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="E1" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>57</v>
+        <v>236</v>
       </c>
       <c r="C3" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>200</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>181</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D5" s="9"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>201</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>202</v>
+        <v>190</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>229</v>
-      </c>
-      <c r="D9" t="s">
-        <v>160</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>120</v>
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>224</v>
+      </c>
+      <c r="D10" t="s">
+        <v>150</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="D11" t="s">
-        <v>159</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>209</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>26</v>
+        <v>238</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>215</v>
-      </c>
-      <c r="E12" t="s">
-        <v>214</v>
+        <v>149</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>222</v>
       </c>
       <c r="D13" t="s">
-        <v>95</v>
+        <v>203</v>
+      </c>
+      <c r="E13" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>14</v>
+        <v>223</v>
       </c>
       <c r="D14" t="s">
-        <v>162</v>
-      </c>
-      <c r="E14" t="s">
-        <v>183</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>201</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>4</v>
+        <v>190</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>175</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>184</v>
+        <v>14</v>
+      </c>
+      <c r="D15" t="s">
+        <v>152</v>
+      </c>
+      <c r="E15" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>200</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>61</v>
+        <v>191</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" t="s">
-        <v>161</v>
+        <v>165</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>159</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>213</v>
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" t="s">
+        <v>151</v>
+      </c>
+      <c r="E17" s="12" t="s">
         <v>201</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="C17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D17" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C18" t="s">
-        <v>99</v>
+        <v>225</v>
       </c>
       <c r="D18" t="s">
-        <v>104</v>
+        <v>88</v>
+      </c>
+      <c r="E18" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>226</v>
       </c>
       <c r="D19" t="s">
-        <v>163</v>
-      </c>
-      <c r="E19" t="s">
-        <v>185</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>178</v>
+        <v>221</v>
       </c>
       <c r="D20" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="E20" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>201</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>7</v>
+        <v>190</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>179</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>171</v>
+        <v>168</v>
+      </c>
+      <c r="D21" t="s">
+        <v>158</v>
       </c>
       <c r="E21" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>197</v>
+        <v>7</v>
+      </c>
+      <c r="C22" t="s">
+        <v>169</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>187</v>
+        <v>161</v>
+      </c>
+      <c r="E22" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>201</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>62</v>
+        <v>190</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>219</v>
       </c>
       <c r="C23" t="s">
-        <v>27</v>
-      </c>
-      <c r="D23" t="s">
-        <v>164</v>
-      </c>
-      <c r="E23" t="s">
-        <v>188</v>
-      </c>
+        <v>187</v>
+      </c>
+      <c r="D23" s="11"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>201</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="C24" t="s">
-        <v>176</v>
-      </c>
-      <c r="D24" t="s">
-        <v>167</v>
-      </c>
-      <c r="E24" t="s">
-        <v>189</v>
+        <v>190</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>205</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>137</v>
+        <v>27</v>
+      </c>
+      <c r="D25" t="s">
+        <v>154</v>
+      </c>
+      <c r="E25" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>63</v>
+        <v>184</v>
       </c>
       <c r="C26" t="s">
-        <v>32</v>
+        <v>166</v>
       </c>
       <c r="D26" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="E26" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>201</v>
-      </c>
-      <c r="B27" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="E27" t="s">
         <v>191</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C27" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D28" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="E28" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>200</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29" t="s">
-        <v>68</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>69</v>
+        <v>191</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>160</v>
       </c>
       <c r="E29" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>125</v>
+        <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>117</v>
+        <v>234</v>
       </c>
       <c r="D30" t="s">
-        <v>118</v>
+        <v>156</v>
+      </c>
+      <c r="E30" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="C31" t="s">
-        <v>210</v>
-      </c>
-      <c r="D31" t="s">
-        <v>219</v>
+        <v>60</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>61</v>
       </c>
       <c r="E31" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B32" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" t="s">
+        <v>227</v>
+      </c>
+      <c r="D32" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>191</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s">
+        <v>228</v>
+      </c>
+      <c r="D33" t="s">
+        <v>207</v>
+      </c>
+      <c r="E33" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>191</v>
+      </c>
+      <c r="B34" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C32" t="s">
-        <v>211</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="C34" t="s">
+        <v>229</v>
+      </c>
+      <c r="D34" t="s">
+        <v>99</v>
+      </c>
+      <c r="E34" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>191</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C35" t="s">
+        <v>231</v>
+      </c>
+      <c r="D35" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>191</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C36" t="s">
+        <v>230</v>
+      </c>
+      <c r="D36" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>191</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C37" t="s">
+        <v>232</v>
+      </c>
+      <c r="D37" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>191</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" t="s">
+        <v>233</v>
+      </c>
+      <c r="D38" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>191</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="C39" t="s">
+        <v>35</v>
+      </c>
+      <c r="D39" t="s">
         <v>107</v>
       </c>
-      <c r="E32" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>201</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="D33" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>201</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="C34" t="s">
-        <v>101</v>
-      </c>
-      <c r="D34" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>201</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="D35" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>201</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D36" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>201</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="D37" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>201</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D38" t="s">
-        <v>216</v>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>191</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C40" t="s">
+        <v>235</v>
+      </c>
+      <c r="D40" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E30">
-    <sortCondition ref="B2:B30"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E32">
+    <sortCondition ref="B2:B32"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="E16" r:id="rId1" xr:uid="{F4F80936-7DCC-48C0-940B-84C684D4BFC4}"/>
-    <hyperlink ref="E5" r:id="rId2" xr:uid="{64B05187-2FCA-467B-A46E-0431E403DB9E}"/>
-    <hyperlink ref="E9" r:id="rId3" xr:uid="{C4CD8744-DE2B-274E-B290-960A5B19E575}"/>
-    <hyperlink ref="E11" r:id="rId4" xr:uid="{BF425982-D1B7-274E-9358-BC78DD6D93C2}"/>
-    <hyperlink ref="E15" r:id="rId5" xr:uid="{37FA49C6-1ACC-C54C-B589-9B635D2542EF}"/>
-    <hyperlink ref="E22" r:id="rId6" xr:uid="{DA33F222-ECA1-2040-8FDF-F138A89BFF19}"/>
+    <hyperlink ref="E17" r:id="rId1" xr:uid="{F4F80936-7DCC-48C0-940B-84C684D4BFC4}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{64B05187-2FCA-467B-A46E-0431E403DB9E}"/>
+    <hyperlink ref="E10" r:id="rId3" xr:uid="{C4CD8744-DE2B-274E-B290-960A5B19E575}"/>
+    <hyperlink ref="E12" r:id="rId4" xr:uid="{BF425982-D1B7-274E-9358-BC78DD6D93C2}"/>
+    <hyperlink ref="E16" r:id="rId5" xr:uid="{37FA49C6-1ACC-C54C-B589-9B635D2542EF}"/>
+    <hyperlink ref="E24" r:id="rId6" xr:uid="{DA33F222-ECA1-2040-8FDF-F138A89BFF19}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId7"/>
@@ -2348,35 +2417,35 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B1" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="C1" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="C2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -2384,10 +2453,10 @@
         <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C4" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -2395,43 +2464,43 @@
         <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C5" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B6" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="C6" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B7" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="C7" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B8" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C8" t="s">
-        <v>230</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -2439,10 +2508,10 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="C9" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -2450,43 +2519,43 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C10" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B11" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="C11" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C12" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B13" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C13" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -2494,55 +2563,55 @@
         <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C14" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="E14" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F14" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="G14" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C15" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B16" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B17" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C17" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="E17" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -2550,38 +2619,38 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="C18" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B19" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C19" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E19" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B20" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C20" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="E20" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2785,15 +2854,15 @@
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{565D9DA6-2D7C-4976-B32E-584E4A2A7F7C}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="aceb4bc4-7be6-4130-8e8a-7008d72bfcc3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="aceb4bc4-7be6-4130-8e8a-7008d72bfcc3"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>